<commit_message>
GF: add product short names + download button inline with title
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gf/20260308_GF_US_Feb-Mar_2026.xlsx
+++ b/gf/20260308_GF_US_Feb-Mar_2026.xlsx
@@ -1600,7 +1600,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -1684,7 +1684,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B6" s="25" t="inlineStr">
@@ -1768,7 +1768,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -1852,7 +1852,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B8" s="25" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -2016,7 +2016,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
@@ -2098,7 +2098,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B12" s="25" t="inlineStr">
@@ -2264,7 +2264,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -2340,7 +2340,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B14" s="25" t="inlineStr">
@@ -2624,7 +2624,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="42" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B4" s="43" t="inlineStr">
@@ -2676,13 +2676,13 @@
         <v>6.684061129110876</v>
       </c>
       <c r="P4" s="48" t="n">
-        <v>0</v>
+        <v>1029.27</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="49" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B5" s="50" t="inlineStr">
@@ -2734,13 +2734,13 @@
         <v>8.440907892529301</v>
       </c>
       <c r="P5" s="55" t="n">
-        <v>0</v>
+        <v>1231.31</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="56" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B6" s="57" t="inlineStr">
@@ -2792,13 +2792,13 @@
         <v>7.995910424466331</v>
       </c>
       <c r="P6" s="62" t="n">
-        <v>0</v>
+        <v>1493.77</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="63" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B7" s="64" t="inlineStr">
@@ -2850,13 +2850,13 @@
         <v>9.601185794663925</v>
       </c>
       <c r="P7" s="69" t="n">
-        <v>0</v>
+        <v>1219.49</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="70" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
@@ -2908,13 +2908,13 @@
         <v>9.849967126890204</v>
       </c>
       <c r="P8" s="76" t="n">
-        <v>0</v>
+        <v>1122.17</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DF7QSTG3 Total</t>
+          <t xml:space="preserve">  ↳ M5 Case Total</t>
         </is>
       </c>
       <c r="B9" s="78" t="inlineStr">
@@ -2969,13 +2969,13 @@
         <v/>
       </c>
       <c r="P9" s="83" t="n">
-        <v>0</v>
+        <v>6096</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="42" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B10" s="43" t="inlineStr">
@@ -3027,13 +3027,13 @@
         <v>0.8093229427325374</v>
       </c>
       <c r="P10" s="48" t="n">
-        <v>0</v>
+        <v>232.03</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="49" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B11" s="50" t="inlineStr">
@@ -3085,13 +3085,13 @@
         <v>1.891802465050872</v>
       </c>
       <c r="P11" s="55" t="n">
-        <v>0</v>
+        <v>200.55</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="56" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B12" s="57" t="inlineStr">
@@ -3143,13 +3143,13 @@
         <v>0.9256959158325417</v>
       </c>
       <c r="P12" s="62" t="n">
-        <v>0</v>
+        <v>227.05</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="63" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B13" s="64" t="inlineStr">
@@ -3201,13 +3201,13 @@
         <v>1.051865332120109</v>
       </c>
       <c r="P13" s="69" t="n">
-        <v>0</v>
+        <v>182.31</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B14" s="71" t="inlineStr">
@@ -3259,13 +3259,13 @@
         <v>0.8153722510411339</v>
       </c>
       <c r="P14" s="76" t="n">
-        <v>0</v>
+        <v>227.05</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DHX988D9 Total</t>
+          <t xml:space="preserve">  ↳ Eskimo Pro 360 Total</t>
         </is>
       </c>
       <c r="B15" s="78" t="inlineStr">
@@ -3320,13 +3320,13 @@
         <v/>
       </c>
       <c r="P15" s="83" t="n">
-        <v>0</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="42" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B16" s="43" t="inlineStr">
@@ -3378,13 +3378,13 @@
         <v>7.119746497665109</v>
       </c>
       <c r="P16" s="48" t="n">
-        <v>0</v>
+        <v>101.63</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="49" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B17" s="50" t="inlineStr">
@@ -3436,13 +3436,13 @@
         <v>15.7640492686682</v>
       </c>
       <c r="P17" s="55" t="n">
-        <v>0</v>
+        <v>88.06999999999999</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="56" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B18" s="57" t="inlineStr">
@@ -3494,13 +3494,13 @@
         <v>8.944380292532719</v>
       </c>
       <c r="P18" s="62" t="n">
-        <v>0</v>
+        <v>176.15</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="63" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B19" s="64" t="inlineStr">
@@ -3552,13 +3552,13 @@
         <v>14.5877378435518</v>
       </c>
       <c r="P19" s="69" t="n">
-        <v>0</v>
+        <v>120.26</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="70" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B20" s="71" t="inlineStr">
@@ -3610,13 +3610,13 @@
         <v>12.19566840926064</v>
       </c>
       <c r="P20" s="76" t="n">
-        <v>0</v>
+        <v>113.48</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DGM9VDFZ Total</t>
+          <t xml:space="preserve">  ↳ M5 Vent Case Total</t>
         </is>
       </c>
       <c r="B21" s="78" t="inlineStr">
@@ -3671,13 +3671,13 @@
         <v/>
       </c>
       <c r="P21" s="83" t="n">
-        <v>0</v>
+        <v>599.6</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="42" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B22" s="43" t="inlineStr">
@@ -3729,13 +3729,13 @@
         <v>2.149643705463183</v>
       </c>
       <c r="P22" s="48" t="n">
-        <v>0</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="49" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B23" s="50" t="inlineStr">
@@ -3787,13 +3787,13 @@
         <v>12.49212260097393</v>
       </c>
       <c r="P23" s="55" t="n">
-        <v>0</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="56" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B24" s="57" t="inlineStr">
@@ -3845,13 +3845,13 @@
         <v>3.046875</v>
       </c>
       <c r="P24" s="62" t="n">
-        <v>0</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="63" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B25" s="64" t="inlineStr">
@@ -3903,13 +3903,13 @@
         <v>7.124132613723979</v>
       </c>
       <c r="P25" s="69" t="n">
-        <v>0</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B26" s="71" t="inlineStr">
@@ -3961,13 +3961,13 @@
         <v>2.744157441574415</v>
       </c>
       <c r="P26" s="76" t="n">
-        <v>0</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DGGX648W Total</t>
+          <t xml:space="preserve">  ↳ S2503 140mm Fan Total</t>
         </is>
       </c>
       <c r="B27" s="78" t="inlineStr">
@@ -4022,13 +4022,13 @@
         <v/>
       </c>
       <c r="P27" s="83" t="n">
-        <v>0</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B28" s="43" t="inlineStr">
@@ -4086,7 +4086,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="49" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B29" s="50" t="inlineStr">
@@ -4138,7 +4138,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="56" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B30" s="57" t="inlineStr">
@@ -4190,7 +4190,7 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="63" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B31" s="64" t="inlineStr">
@@ -4248,7 +4248,7 @@
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="70" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B32" s="71" t="inlineStr">
@@ -4306,7 +4306,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B09X1KD6NH Total</t>
+          <t xml:space="preserve">  ↳ M8 Case Total</t>
         </is>
       </c>
       <c r="B33" s="78" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="42" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B34" s="43" t="inlineStr">
@@ -4425,7 +4425,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="49" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B35" s="50" t="inlineStr">
@@ -4477,7 +4477,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="56" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B36" s="57" t="inlineStr">
@@ -4535,7 +4535,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="63" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B37" s="64" t="inlineStr">
@@ -4593,7 +4593,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="70" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B38" s="71" t="inlineStr">
@@ -4651,7 +4651,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DJ2X2SK8 Total</t>
+          <t xml:space="preserve">  ↳ S2503 120mm Fan Total</t>
         </is>
       </c>
       <c r="B39" s="78" t="inlineStr">
@@ -4712,7 +4712,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="42" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B40" s="43" t="inlineStr">
@@ -4764,7 +4764,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="49" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B41" s="50" t="inlineStr">
@@ -4822,7 +4822,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="56" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B42" s="57" t="inlineStr">
@@ -4880,7 +4880,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="63" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B43" s="64" t="inlineStr">
@@ -4938,7 +4938,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="70" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B44" s="71" t="inlineStr">
@@ -4996,7 +4996,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0CKWQX52V Total</t>
+          <t xml:space="preserve">  ↳ M4 King Arthur Total</t>
         </is>
       </c>
       <c r="B45" s="78" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="42" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B46" s="43" t="inlineStr">
@@ -5109,13 +5109,13 @@
         <v>15.07537688442211</v>
       </c>
       <c r="P46" s="48" t="n">
-        <v>0</v>
+        <v>4.97</v>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="49" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B47" s="50" t="inlineStr">
@@ -5167,13 +5167,13 @@
         <v>42.8643216080402</v>
       </c>
       <c r="P47" s="55" t="n">
-        <v>0</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="56" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B48" s="57" t="inlineStr">
@@ -5225,13 +5225,13 @@
         <v>15.74539363484087</v>
       </c>
       <c r="P48" s="62" t="n">
-        <v>0</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="63" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B49" s="64" t="inlineStr">
@@ -5283,13 +5283,13 @@
         <v>55.77889447236181</v>
       </c>
       <c r="P49" s="69" t="n">
-        <v>0</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="70" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B50" s="71" t="inlineStr">
@@ -5341,13 +5341,13 @@
         <v>33.61809045226131</v>
       </c>
       <c r="P50" s="76" t="n">
-        <v>0</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0CRTD8V77 Total</t>
+          <t xml:space="preserve">  ↳ S2503R 120mm Fan Total</t>
         </is>
       </c>
       <c r="B51" s="78" t="inlineStr">
@@ -5402,13 +5402,13 @@
         <v/>
       </c>
       <c r="P51" s="83" t="n">
-        <v>0</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="42" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B52" s="43" t="inlineStr">
@@ -5460,7 +5460,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="49" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B53" s="50" t="inlineStr">
@@ -5512,7 +5512,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="56" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B54" s="57" t="inlineStr">
@@ -5570,7 +5570,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="63" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B55" s="64" t="inlineStr">
@@ -5622,7 +5622,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="70" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B56" s="71" t="inlineStr">
@@ -5674,7 +5674,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B0DHZ1GPXB Total</t>
+          <t xml:space="preserve">  ↳ S3805 Fan Total</t>
         </is>
       </c>
       <c r="B57" s="78" t="inlineStr">
@@ -5735,7 +5735,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="42" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B58" s="43" t="inlineStr">
@@ -5787,7 +5787,7 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="49" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B59" s="50" t="inlineStr">
@@ -5839,7 +5839,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="56" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B60" s="57" t="inlineStr">
@@ -5891,7 +5891,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="63" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B61" s="64" t="inlineStr">
@@ -5943,7 +5943,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="70" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B62" s="71" t="inlineStr">
@@ -5995,7 +5995,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ B09X697T7N Total</t>
+          <t xml:space="preserve">  ↳ M6 Case Total</t>
         </is>
       </c>
       <c r="B63" s="78" t="inlineStr">
@@ -6164,7 +6164,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B4" s="43" t="inlineStr">
@@ -6213,7 +6213,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B5" s="50" t="inlineStr">
@@ -6262,7 +6262,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B6" s="57" t="inlineStr">
@@ -6311,7 +6311,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B7" s="64" t="inlineStr">
@@ -6360,7 +6360,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
@@ -6409,7 +6409,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B9" s="43" t="inlineStr">
@@ -6458,7 +6458,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B10" s="50" t="inlineStr">
@@ -6507,7 +6507,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B11" s="57" t="inlineStr">
@@ -6556,7 +6556,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B12" s="64" t="inlineStr">
@@ -6605,7 +6605,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B13" s="71" t="inlineStr">
@@ -6654,7 +6654,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B14" s="43" t="inlineStr">
@@ -6703,7 +6703,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B15" s="50" t="inlineStr">
@@ -6752,7 +6752,7 @@
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B16" s="57" t="inlineStr">
@@ -6801,7 +6801,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B17" s="64" t="inlineStr">
@@ -6850,7 +6850,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B18" s="71" t="inlineStr">
@@ -6899,7 +6899,7 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B19" s="43" t="inlineStr">
@@ -6948,7 +6948,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B20" s="50" t="inlineStr">
@@ -6997,7 +6997,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B21" s="57" t="inlineStr">
@@ -7046,7 +7046,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B22" s="64" t="inlineStr">
@@ -7095,7 +7095,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B23" s="71" t="inlineStr">
@@ -7144,7 +7144,7 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B24" s="43" t="inlineStr">
@@ -7193,7 +7193,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B25" s="50" t="inlineStr">
@@ -7242,7 +7242,7 @@
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B26" s="57" t="inlineStr">
@@ -7291,7 +7291,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B27" s="64" t="inlineStr">
@@ -7340,7 +7340,7 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B28" s="71" t="inlineStr">
@@ -7389,7 +7389,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B29" s="43" t="inlineStr">
@@ -7438,7 +7438,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B30" s="50" t="inlineStr">
@@ -7483,7 +7483,7 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B31" s="57" t="inlineStr">
@@ -7532,7 +7532,7 @@
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B32" s="64" t="inlineStr">
@@ -7581,7 +7581,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B33" s="71" t="inlineStr">
@@ -7630,7 +7630,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B34" s="43" t="inlineStr">
@@ -7679,7 +7679,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B35" s="50" t="inlineStr">
@@ -7728,7 +7728,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B36" s="57" t="inlineStr">
@@ -7777,7 +7777,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B37" s="64" t="inlineStr">
@@ -7826,7 +7826,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B38" s="71" t="inlineStr">
@@ -7871,7 +7871,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B39" s="43" t="inlineStr">
@@ -7920,7 +7920,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B40" s="50" t="inlineStr">
@@ -7965,7 +7965,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B41" s="57" t="inlineStr">
@@ -8010,7 +8010,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B42" s="64" t="inlineStr">
@@ -8059,7 +8059,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B43" s="71" t="inlineStr">
@@ -8108,7 +8108,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="94" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B44" s="43" t="inlineStr">
@@ -8157,7 +8157,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="97" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B45" s="50" t="inlineStr">
@@ -8202,7 +8202,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="100" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B46" s="57" t="inlineStr">
@@ -8251,7 +8251,7 @@
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="103" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B47" s="64" t="inlineStr">
@@ -8300,7 +8300,7 @@
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="106" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B48" s="71" t="inlineStr">
@@ -8349,7 +8349,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="94" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B49" s="43" t="inlineStr">
@@ -8398,7 +8398,7 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="97" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B50" s="50" t="inlineStr">
@@ -8447,7 +8447,7 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="100" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B51" s="57" t="inlineStr">
@@ -8496,7 +8496,7 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="103" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B52" s="64" t="inlineStr">
@@ -8545,7 +8545,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="106" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B53" s="71" t="inlineStr">
@@ -8594,7 +8594,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="94" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B54" s="43" t="inlineStr">
@@ -8639,7 +8639,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="97" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B55" s="50" t="inlineStr">
@@ -8688,7 +8688,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="100" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B56" s="57" t="inlineStr">
@@ -8737,7 +8737,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="103" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B57" s="64" t="inlineStr">
@@ -8786,7 +8786,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="106" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B58" s="71" t="inlineStr">
@@ -8835,7 +8835,7 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="94" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B59" s="43" t="inlineStr">
@@ -8884,7 +8884,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="97" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B60" s="50" t="inlineStr">
@@ -8929,7 +8929,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="100" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B61" s="57" t="inlineStr">
@@ -8978,7 +8978,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="103" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B62" s="64" t="inlineStr">
@@ -9023,7 +9023,7 @@
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="106" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B63" s="71" t="inlineStr">
@@ -9072,7 +9072,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="94" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B64" s="43" t="inlineStr">
@@ -9117,7 +9117,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="97" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B65" s="50" t="inlineStr">
@@ -9162,7 +9162,7 @@
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="100" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B66" s="57" t="inlineStr">
@@ -9207,7 +9207,7 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="103" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B67" s="64" t="inlineStr">
@@ -9252,7 +9252,7 @@
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="106" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B68" s="71" t="inlineStr">
@@ -9297,7 +9297,7 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B69" s="43" t="inlineStr">
@@ -9346,7 +9346,7 @@
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B70" s="50" t="inlineStr">
@@ -9395,7 +9395,7 @@
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B71" s="57" t="inlineStr">
@@ -9444,7 +9444,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B72" s="64" t="inlineStr">
@@ -9493,7 +9493,7 @@
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B73" s="71" t="inlineStr">
@@ -9542,7 +9542,7 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B74" s="43" t="inlineStr">
@@ -9591,7 +9591,7 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B75" s="50" t="inlineStr">
@@ -9640,7 +9640,7 @@
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B76" s="57" t="inlineStr">
@@ -9689,7 +9689,7 @@
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B77" s="64" t="inlineStr">
@@ -9738,7 +9738,7 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B78" s="71" t="inlineStr">
@@ -9787,7 +9787,7 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B79" s="43" t="inlineStr">
@@ -9832,7 +9832,7 @@
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B80" s="50" t="inlineStr">
@@ -9881,7 +9881,7 @@
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B81" s="57" t="inlineStr">
@@ -9930,7 +9930,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B82" s="64" t="inlineStr">
@@ -9979,7 +9979,7 @@
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B83" s="71" t="inlineStr">
@@ -10028,7 +10028,7 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B84" s="43" t="inlineStr">
@@ -10073,7 +10073,7 @@
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B85" s="50" t="inlineStr">
@@ -10118,7 +10118,7 @@
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B86" s="57" t="inlineStr">
@@ -10167,7 +10167,7 @@
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B87" s="64" t="inlineStr">
@@ -10212,7 +10212,7 @@
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B88" s="71" t="inlineStr">
@@ -10261,7 +10261,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B89" s="43" t="inlineStr">
@@ -10306,7 +10306,7 @@
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B90" s="50" t="inlineStr">
@@ -10351,7 +10351,7 @@
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B91" s="57" t="inlineStr">
@@ -10396,7 +10396,7 @@
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B92" s="64" t="inlineStr">
@@ -10441,7 +10441,7 @@
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B93" s="71" t="inlineStr">
@@ -10486,7 +10486,7 @@
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="94" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B94" s="43" t="inlineStr">
@@ -10531,7 +10531,7 @@
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="97" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B95" s="50" t="inlineStr">
@@ -10576,7 +10576,7 @@
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="100" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B96" s="57" t="inlineStr">
@@ -10621,7 +10621,7 @@
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="103" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B97" s="64" t="inlineStr">
@@ -10666,7 +10666,7 @@
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="106" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B98" s="71" t="inlineStr">
@@ -10711,7 +10711,7 @@
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B99" s="43" t="inlineStr">
@@ -10760,7 +10760,7 @@
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B100" s="50" t="inlineStr">
@@ -10809,7 +10809,7 @@
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B101" s="57" t="inlineStr">
@@ -10858,7 +10858,7 @@
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B102" s="64" t="inlineStr">
@@ -10907,7 +10907,7 @@
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B103" s="71" t="inlineStr">
@@ -10956,7 +10956,7 @@
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B104" s="43" t="inlineStr">
@@ -11005,7 +11005,7 @@
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B105" s="50" t="inlineStr">
@@ -11054,7 +11054,7 @@
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B106" s="57" t="inlineStr">
@@ -11103,7 +11103,7 @@
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B107" s="64" t="inlineStr">
@@ -11152,7 +11152,7 @@
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B108" s="71" t="inlineStr">
@@ -11201,7 +11201,7 @@
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B109" s="43" t="inlineStr">
@@ -11250,7 +11250,7 @@
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B110" s="50" t="inlineStr">
@@ -11299,7 +11299,7 @@
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B111" s="57" t="inlineStr">
@@ -11344,7 +11344,7 @@
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B112" s="64" t="inlineStr">
@@ -11389,7 +11389,7 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B113" s="71" t="inlineStr">
@@ -11438,7 +11438,7 @@
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B114" s="43" t="inlineStr">
@@ -11483,7 +11483,7 @@
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B115" s="50" t="inlineStr">
@@ -11528,7 +11528,7 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B116" s="57" t="inlineStr">
@@ -11577,7 +11577,7 @@
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B117" s="64" t="inlineStr">
@@ -11622,7 +11622,7 @@
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B118" s="71" t="inlineStr">
@@ -11671,7 +11671,7 @@
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B119" s="43" t="inlineStr">
@@ -11720,7 +11720,7 @@
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B120" s="50" t="inlineStr">
@@ -11769,7 +11769,7 @@
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B121" s="57" t="inlineStr">
@@ -11818,7 +11818,7 @@
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B122" s="64" t="inlineStr">
@@ -11863,7 +11863,7 @@
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B123" s="71" t="inlineStr">
@@ -11912,7 +11912,7 @@
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B124" s="43" t="inlineStr">
@@ -11957,7 +11957,7 @@
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B125" s="50" t="inlineStr">
@@ -12002,7 +12002,7 @@
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B126" s="57" t="inlineStr">
@@ -12051,7 +12051,7 @@
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B127" s="64" t="inlineStr">
@@ -12100,7 +12100,7 @@
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B128" s="71" t="inlineStr">
@@ -12149,7 +12149,7 @@
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B129" s="43" t="inlineStr">
@@ -12198,7 +12198,7 @@
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B130" s="50" t="inlineStr">
@@ -12247,7 +12247,7 @@
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B131" s="57" t="inlineStr">
@@ -12296,7 +12296,7 @@
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B132" s="64" t="inlineStr">
@@ -12341,7 +12341,7 @@
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B133" s="71" t="inlineStr">
@@ -12390,7 +12390,7 @@
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="94" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B134" s="43" t="inlineStr">
@@ -12439,7 +12439,7 @@
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="97" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B135" s="50" t="inlineStr">
@@ -12484,7 +12484,7 @@
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="100" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B136" s="57" t="inlineStr">
@@ -12529,7 +12529,7 @@
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="103" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B137" s="64" t="inlineStr">
@@ -12574,7 +12574,7 @@
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="106" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B138" s="71" t="inlineStr">
@@ -12623,7 +12623,7 @@
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="94" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B139" s="43" t="inlineStr">
@@ -12672,7 +12672,7 @@
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="97" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B140" s="50" t="inlineStr">
@@ -12717,7 +12717,7 @@
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="100" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B141" s="57" t="inlineStr">
@@ -12762,7 +12762,7 @@
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="103" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B142" s="64" t="inlineStr">
@@ -12811,7 +12811,7 @@
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="106" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B143" s="71" t="inlineStr">
@@ -12860,7 +12860,7 @@
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="94" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B144" s="43" t="inlineStr">
@@ -12905,7 +12905,7 @@
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="97" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B145" s="50" t="inlineStr">
@@ -12950,7 +12950,7 @@
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="100" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B146" s="57" t="inlineStr">
@@ -12995,7 +12995,7 @@
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="103" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B147" s="64" t="inlineStr">
@@ -13040,7 +13040,7 @@
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="106" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B148" s="71" t="inlineStr">
@@ -13089,7 +13089,7 @@
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="94" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B149" s="43" t="inlineStr">
@@ -13134,7 +13134,7 @@
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="97" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B150" s="50" t="inlineStr">
@@ -13179,7 +13179,7 @@
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="100" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B151" s="57" t="inlineStr">
@@ -13224,7 +13224,7 @@
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="103" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B152" s="64" t="inlineStr">
@@ -13269,7 +13269,7 @@
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="106" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B153" s="71" t="inlineStr">
@@ -13314,7 +13314,7 @@
     <row r="154" ht="16" customHeight="1">
       <c r="A154" s="94" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B154" s="43" t="inlineStr">
@@ -13359,7 +13359,7 @@
     <row r="155" ht="16" customHeight="1">
       <c r="A155" s="97" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B155" s="50" t="inlineStr">
@@ -13404,7 +13404,7 @@
     <row r="156" ht="16" customHeight="1">
       <c r="A156" s="100" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B156" s="57" t="inlineStr">
@@ -13451,7 +13451,7 @@
     <row r="157" ht="16" customHeight="1">
       <c r="A157" s="103" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B157" s="64" t="inlineStr">
@@ -13498,7 +13498,7 @@
     <row r="158" ht="16" customHeight="1">
       <c r="A158" s="106" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B158" s="71" t="inlineStr">
@@ -13547,7 +13547,7 @@
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="94" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B159" s="43" t="inlineStr">
@@ -13594,7 +13594,7 @@
     <row r="160" ht="16" customHeight="1">
       <c r="A160" s="97" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B160" s="50" t="inlineStr">
@@ -13639,7 +13639,7 @@
     <row r="161" ht="16" customHeight="1">
       <c r="A161" s="100" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B161" s="57" t="inlineStr">
@@ -13684,7 +13684,7 @@
     <row r="162" ht="16" customHeight="1">
       <c r="A162" s="103" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B162" s="64" t="inlineStr">
@@ -13731,7 +13731,7 @@
     <row r="163" ht="16" customHeight="1">
       <c r="A163" s="106" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B163" s="71" t="inlineStr">
@@ -13778,7 +13778,7 @@
     <row r="164" ht="16" customHeight="1">
       <c r="A164" s="94" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B164" s="43" t="inlineStr">
@@ -13823,7 +13823,7 @@
     <row r="165" ht="16" customHeight="1">
       <c r="A165" s="97" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B165" s="50" t="inlineStr">
@@ -13868,7 +13868,7 @@
     <row r="166" ht="16" customHeight="1">
       <c r="A166" s="100" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B166" s="57" t="inlineStr">
@@ -13913,7 +13913,7 @@
     <row r="167" ht="16" customHeight="1">
       <c r="A167" s="103" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B167" s="64" t="inlineStr">
@@ -13958,7 +13958,7 @@
     <row r="168" ht="16" customHeight="1">
       <c r="A168" s="106" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B168" s="71" t="inlineStr">
@@ -14003,7 +14003,7 @@
     <row r="169" ht="16" customHeight="1">
       <c r="A169" s="94" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B169" s="43" t="inlineStr">
@@ -14048,7 +14048,7 @@
     <row r="170" ht="16" customHeight="1">
       <c r="A170" s="97" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B170" s="50" t="inlineStr">
@@ -14097,7 +14097,7 @@
     <row r="171" ht="16" customHeight="1">
       <c r="A171" s="100" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B171" s="57" t="inlineStr">
@@ -14142,7 +14142,7 @@
     <row r="172" ht="16" customHeight="1">
       <c r="A172" s="103" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B172" s="64" t="inlineStr">
@@ -14191,7 +14191,7 @@
     <row r="173" ht="16" customHeight="1">
       <c r="A173" s="106" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B173" s="71" t="inlineStr">
@@ -14236,7 +14236,7 @@
     <row r="174" ht="16" customHeight="1">
       <c r="A174" s="94" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B174" s="43" t="inlineStr">
@@ -14281,7 +14281,7 @@
     <row r="175" ht="16" customHeight="1">
       <c r="A175" s="97" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B175" s="50" t="inlineStr">
@@ -14326,7 +14326,7 @@
     <row r="176" ht="16" customHeight="1">
       <c r="A176" s="100" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B176" s="57" t="inlineStr">
@@ -14375,7 +14375,7 @@
     <row r="177" ht="16" customHeight="1">
       <c r="A177" s="103" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B177" s="64" t="inlineStr">
@@ -14420,7 +14420,7 @@
     <row r="178" ht="16" customHeight="1">
       <c r="A178" s="106" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B178" s="71" t="inlineStr">
@@ -14469,7 +14469,7 @@
     <row r="179" ht="16" customHeight="1">
       <c r="A179" s="94" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B179" s="43" t="inlineStr">
@@ -14514,7 +14514,7 @@
     <row r="180" ht="16" customHeight="1">
       <c r="A180" s="97" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B180" s="50" t="inlineStr">
@@ -14559,7 +14559,7 @@
     <row r="181" ht="16" customHeight="1">
       <c r="A181" s="100" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B181" s="57" t="inlineStr">
@@ -14604,7 +14604,7 @@
     <row r="182" ht="16" customHeight="1">
       <c r="A182" s="103" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B182" s="64" t="inlineStr">
@@ -14649,7 +14649,7 @@
     <row r="183" ht="16" customHeight="1">
       <c r="A183" s="106" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B183" s="71" t="inlineStr">
@@ -14694,7 +14694,7 @@
     <row r="184" ht="16" customHeight="1">
       <c r="A184" s="94" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B184" s="43" t="inlineStr">
@@ -14743,7 +14743,7 @@
     <row r="185" ht="16" customHeight="1">
       <c r="A185" s="97" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B185" s="50" t="inlineStr">
@@ -14792,7 +14792,7 @@
     <row r="186" ht="16" customHeight="1">
       <c r="A186" s="100" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B186" s="57" t="inlineStr">
@@ -14841,7 +14841,7 @@
     <row r="187" ht="16" customHeight="1">
       <c r="A187" s="103" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B187" s="64" t="inlineStr">
@@ -14890,7 +14890,7 @@
     <row r="188" ht="16" customHeight="1">
       <c r="A188" s="106" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B188" s="71" t="inlineStr">
@@ -14939,7 +14939,7 @@
     <row r="189" ht="16" customHeight="1">
       <c r="A189" s="94" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B189" s="43" t="inlineStr">
@@ -14984,7 +14984,7 @@
     <row r="190" ht="16" customHeight="1">
       <c r="A190" s="97" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B190" s="50" t="inlineStr">
@@ -15029,7 +15029,7 @@
     <row r="191" ht="16" customHeight="1">
       <c r="A191" s="100" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B191" s="57" t="inlineStr">
@@ -15078,7 +15078,7 @@
     <row r="192" ht="16" customHeight="1">
       <c r="A192" s="103" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B192" s="64" t="inlineStr">
@@ -15123,7 +15123,7 @@
     <row r="193" ht="16" customHeight="1">
       <c r="A193" s="106" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B193" s="71" t="inlineStr">
@@ -15168,7 +15168,7 @@
     <row r="194" ht="16" customHeight="1">
       <c r="A194" s="94" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B194" s="43" t="inlineStr">
@@ -15213,7 +15213,7 @@
     <row r="195" ht="16" customHeight="1">
       <c r="A195" s="97" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B195" s="50" t="inlineStr">
@@ -15258,7 +15258,7 @@
     <row r="196" ht="16" customHeight="1">
       <c r="A196" s="100" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B196" s="57" t="inlineStr">
@@ -15303,7 +15303,7 @@
     <row r="197" ht="16" customHeight="1">
       <c r="A197" s="103" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B197" s="64" t="inlineStr">
@@ -15348,7 +15348,7 @@
     <row r="198" ht="16" customHeight="1">
       <c r="A198" s="106" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B198" s="71" t="inlineStr">
@@ -15539,7 +15539,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="B5" s="122" t="inlineStr">
@@ -15719,7 +15719,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="B9" s="122" t="inlineStr">
@@ -15899,7 +15899,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="B13" s="122" t="inlineStr">
@@ -16079,7 +16079,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="B17" s="122" t="inlineStr">
@@ -16259,7 +16259,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="B21" s="122" t="inlineStr">
@@ -16427,7 +16427,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="B25" s="122" t="inlineStr">
@@ -16601,7 +16601,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="B29" s="122" t="inlineStr">
@@ -16775,7 +16775,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="B33" s="122" t="inlineStr">
@@ -16955,7 +16955,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="B37" s="122" t="inlineStr">
@@ -17115,7 +17115,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>B09X697T7N</t>
+          <t>M6 Case</t>
         </is>
       </c>
       <c r="B41" s="122" t="inlineStr">
@@ -20268,7 +20268,7 @@
       </c>
       <c r="B7" s="177" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="C7" s="178" t="inlineStr">
@@ -20292,7 +20292,7 @@
         <v>39.13289294734797</v>
       </c>
       <c r="I7" s="183" t="n">
-        <v>0</v>
+        <v>6096</v>
       </c>
       <c r="J7" s="184" t="inlineStr">
         <is>
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B8" s="177" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="C8" s="178" t="inlineStr">
@@ -20337,7 +20337,7 @@
         <v>5.259957256654362</v>
       </c>
       <c r="I8" s="183" t="n">
-        <v>0</v>
+        <v>1069</v>
       </c>
       <c r="J8" s="184" t="inlineStr">
         <is>
@@ -20358,7 +20358,7 @@
       </c>
       <c r="B9" s="177" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="C9" s="178" t="inlineStr">
@@ -20382,7 +20382,7 @@
         <v>1.989119875655722</v>
       </c>
       <c r="I9" s="183" t="n">
-        <v>0</v>
+        <v>14.9</v>
       </c>
       <c r="J9" s="184" t="inlineStr">
         <is>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B11" s="188" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="C11" s="189" t="inlineStr">
@@ -20434,7 +20434,7 @@
         <v>2.436370701379444</v>
       </c>
       <c r="I11" s="194" t="n">
-        <v>0</v>
+        <v>599.6</v>
       </c>
       <c r="J11" s="195" t="inlineStr">
         <is>
@@ -20455,7 +20455,7 @@
       </c>
       <c r="B12" s="188" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="C12" s="189" t="inlineStr">
@@ -20507,7 +20507,7 @@
       </c>
       <c r="B14" s="200" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="C14" s="201" t="inlineStr">
@@ -20552,7 +20552,7 @@
       </c>
       <c r="B15" s="200" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="C15" s="201" t="inlineStr">
@@ -20576,7 +20576,7 @@
         <v>-0.8453468039634738</v>
       </c>
       <c r="I15" s="206" t="n">
-        <v>0</v>
+        <v>19.9</v>
       </c>
       <c r="J15" s="207" t="inlineStr">
         <is>
@@ -20597,7 +20597,7 @@
       </c>
       <c r="B16" s="200" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="C16" s="201" t="inlineStr">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B18" s="211" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="C18" s="212" t="inlineStr">
@@ -20783,7 +20783,7 @@
       <c r="A5" s="220" t="inlineStr"/>
       <c r="B5" s="177" t="inlineStr">
         <is>
-          <t>B0DF7QSTG3</t>
+          <t>M5 Case</t>
         </is>
       </c>
       <c r="C5" s="176" t="inlineStr">
@@ -20881,7 +20881,7 @@
       <c r="A10" s="220" t="inlineStr"/>
       <c r="B10" s="177" t="inlineStr">
         <is>
-          <t>B0DHX988D9</t>
+          <t>Eskimo Pro 360</t>
         </is>
       </c>
       <c r="C10" s="176" t="inlineStr">
@@ -20979,7 +20979,7 @@
       <c r="A15" s="220" t="inlineStr"/>
       <c r="B15" s="177" t="inlineStr">
         <is>
-          <t>B0DGGX648W</t>
+          <t>S2503 140mm Fan</t>
         </is>
       </c>
       <c r="C15" s="176" t="inlineStr">
@@ -21084,7 +21084,7 @@
       <c r="A21" s="224" t="inlineStr"/>
       <c r="B21" s="188" t="inlineStr">
         <is>
-          <t>B0DGM9VDFZ</t>
+          <t>M5 Vent Case</t>
         </is>
       </c>
       <c r="C21" s="187" t="inlineStr">
@@ -21182,7 +21182,7 @@
       <c r="A26" s="224" t="inlineStr"/>
       <c r="B26" s="188" t="inlineStr">
         <is>
-          <t>B09X1KD6NH</t>
+          <t>M8 Case</t>
         </is>
       </c>
       <c r="C26" s="187" t="inlineStr">
@@ -21287,7 +21287,7 @@
       <c r="A32" s="227" t="inlineStr"/>
       <c r="B32" s="200" t="inlineStr">
         <is>
-          <t>B0CKWQX52V</t>
+          <t>M4 King Arthur</t>
         </is>
       </c>
       <c r="C32" s="199" t="inlineStr">
@@ -21385,7 +21385,7 @@
       <c r="A37" s="227" t="inlineStr"/>
       <c r="B37" s="200" t="inlineStr">
         <is>
-          <t>B0CRTD8V77</t>
+          <t>S2503R 120mm Fan</t>
         </is>
       </c>
       <c r="C37" s="199" t="inlineStr">
@@ -21483,7 +21483,7 @@
       <c r="A42" s="227" t="inlineStr"/>
       <c r="B42" s="200" t="inlineStr">
         <is>
-          <t>B0DHZ1GPXB</t>
+          <t>S3805 Fan</t>
         </is>
       </c>
       <c r="C42" s="199" t="inlineStr">
@@ -21588,7 +21588,7 @@
       <c r="A48" s="230" t="inlineStr"/>
       <c r="B48" s="211" t="inlineStr">
         <is>
-          <t>B0DJ2X2SK8</t>
+          <t>S2503 120mm Fan</t>
         </is>
       </c>
       <c r="C48" s="210" t="inlineStr">

</xml_diff>